<commit_message>
Updated of smtpage 7tnthebrew
</commit_message>
<xml_diff>
--- a/sampledata/RLLT-Tabledata_updated.xlsx
+++ b/sampledata/RLLT-Tabledata_updated.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="I:\RLLT\Webapp\sampledata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBC9DEA6-9571-42D1-9257-9A62D5F5BA97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31BA0B62-9B38-4952-98A4-502F3646C44C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="43">
   <si>
     <t>Module</t>
   </si>
@@ -126,9 +126,6 @@
     <t>23min</t>
   </si>
   <si>
-    <t>55min</t>
-  </si>
-  <si>
     <r>
       <rPr>
         <b/>
@@ -165,28 +162,6 @@
     <r>
       <rPr>
         <b/>
-        <sz val="7.5"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>PRO</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="7.5"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>PSA</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
         <sz val="6.5"/>
         <rFont val="Arial"/>
         <family val="2"/>
@@ -279,19 +254,14 @@
         <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
-      <t>`1530</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="6.5"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
       <t>1+</t>
     </r>
+  </si>
+  <si>
+    <t>PRO</t>
+  </si>
+  <si>
+    <t>PSA</t>
   </si>
 </sst>
 </file>
@@ -405,7 +375,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -430,6 +400,9 @@
       <alignment horizontal="center" vertical="top" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -707,54 +680,98 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:O42"/>
+  <dimension ref="B1:O41"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
     <col min="7" max="7" width="13.77734375" customWidth="1"/>
   </cols>
   <sheetData>
+    <row r="1" spans="2:15">
+      <c r="B1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="K1" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="L1" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="M1" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="N1" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="O1" s="6" t="s">
+        <v>34</v>
+      </c>
+    </row>
     <row r="2" spans="2:15">
-      <c r="B2" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F2" s="2" t="s">
+      <c r="B2" s="1">
+        <v>1</v>
+      </c>
+      <c r="C2" s="3">
+        <v>1</v>
+      </c>
+      <c r="D2" s="3">
+        <v>6</v>
+      </c>
+      <c r="E2" s="3">
+        <v>180</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="G2" s="3">
+        <v>30</v>
+      </c>
+      <c r="H2" s="8">
+        <v>12</v>
+      </c>
+      <c r="I2" s="8">
         <v>4</v>
       </c>
-      <c r="G2" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="H2" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="I2" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="J2" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="K2" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="L2" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="M2" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="N2" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="O2" s="6" t="s">
-        <v>37</v>
+      <c r="J2" s="8">
+        <v>6</v>
+      </c>
+      <c r="K2" s="8">
+        <v>6</v>
+      </c>
+      <c r="L2" s="8">
+        <v>6</v>
+      </c>
+      <c r="M2" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="N2" s="8">
+        <v>14977</v>
+      </c>
+      <c r="O2" s="8">
+        <v>180</v>
       </c>
     </row>
     <row r="3" spans="2:15">
@@ -762,22 +779,22 @@
         <v>1</v>
       </c>
       <c r="C3" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D3" s="3">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E3" s="3">
-        <v>180</v>
+        <v>30</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G3" s="3">
         <v>30</v>
       </c>
-      <c r="H3" s="8">
-        <v>12</v>
+      <c r="H3" s="9" t="s">
+        <v>35</v>
       </c>
       <c r="I3" s="8">
         <v>4</v>
@@ -786,19 +803,19 @@
         <v>6</v>
       </c>
       <c r="K3" s="8">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="L3" s="8">
-        <v>6</v>
-      </c>
-      <c r="M3" s="9" t="s">
-        <v>42</v>
+        <v>1</v>
+      </c>
+      <c r="M3" s="8">
+        <v>227</v>
       </c>
       <c r="N3" s="8">
-        <v>14977</v>
+        <v>7375</v>
       </c>
       <c r="O3" s="8">
-        <v>180</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4" spans="2:15">
@@ -806,7 +823,7 @@
         <v>1</v>
       </c>
       <c r="C4" s="3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D4" s="3">
         <v>1</v>
@@ -815,16 +832,16 @@
         <v>30</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G4" s="3">
         <v>30</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="I4" s="8">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="J4" s="8">
         <v>6</v>
@@ -836,10 +853,10 @@
         <v>1</v>
       </c>
       <c r="M4" s="8">
-        <v>227</v>
+        <v>341</v>
       </c>
       <c r="N4" s="8">
-        <v>7375</v>
+        <v>7619</v>
       </c>
       <c r="O4" s="8">
         <v>30</v>
@@ -850,7 +867,7 @@
         <v>1</v>
       </c>
       <c r="C5" s="3">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D5" s="3">
         <v>1</v>
@@ -859,16 +876,16 @@
         <v>30</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G5" s="3">
         <v>30</v>
       </c>
       <c r="H5" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="I5" s="8">
-        <v>19</v>
+        <v>37</v>
+      </c>
+      <c r="I5" s="9" t="s">
+        <v>38</v>
       </c>
       <c r="J5" s="8">
         <v>6</v>
@@ -880,10 +897,10 @@
         <v>1</v>
       </c>
       <c r="M5" s="8">
-        <v>341</v>
+        <v>312</v>
       </c>
       <c r="N5" s="8">
-        <v>7619</v>
+        <v>8275</v>
       </c>
       <c r="O5" s="8">
         <v>30</v>
@@ -894,7 +911,7 @@
         <v>1</v>
       </c>
       <c r="C6" s="3">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D6" s="3">
         <v>1</v>
@@ -903,16 +920,16 @@
         <v>30</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G6" s="3">
         <v>30</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="I6" s="9" t="s">
-        <v>41</v>
+        <v>36</v>
+      </c>
+      <c r="I6" s="8">
+        <v>19</v>
       </c>
       <c r="J6" s="8">
         <v>6</v>
@@ -924,10 +941,10 @@
         <v>1</v>
       </c>
       <c r="M6" s="8">
-        <v>312</v>
+        <v>433</v>
       </c>
       <c r="N6" s="8">
-        <v>8275</v>
+        <v>11917</v>
       </c>
       <c r="O6" s="8">
         <v>30</v>
@@ -935,10 +952,10 @@
     </row>
     <row r="7" spans="2:15">
       <c r="B7" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C7" s="3">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D7" s="3">
         <v>1</v>
@@ -947,16 +964,16 @@
         <v>30</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="G7" s="3">
         <v>30</v>
       </c>
-      <c r="H7" s="9" t="s">
-        <v>39</v>
+      <c r="H7" s="8">
+        <v>1</v>
       </c>
       <c r="I7" s="8">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="J7" s="8">
         <v>6</v>
@@ -968,10 +985,10 @@
         <v>1</v>
       </c>
       <c r="M7" s="8">
-        <v>433</v>
+        <v>1189</v>
       </c>
       <c r="N7" s="8">
-        <v>11917</v>
+        <v>31102</v>
       </c>
       <c r="O7" s="8">
         <v>30</v>
@@ -982,16 +999,16 @@
         <v>2</v>
       </c>
       <c r="C8" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D8" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E8" s="3">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="G8" s="3">
         <v>30</v>
@@ -1003,22 +1020,22 @@
         <v>1</v>
       </c>
       <c r="J8" s="8">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="K8" s="8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L8" s="8">
         <v>1</v>
       </c>
       <c r="M8" s="8">
-        <v>1189</v>
+        <v>1220</v>
       </c>
       <c r="N8" s="8">
-        <v>31102</v>
+        <v>32017</v>
       </c>
       <c r="O8" s="8">
-        <v>30</v>
+        <v>60</v>
       </c>
     </row>
     <row r="9" spans="2:15">
@@ -1026,16 +1043,16 @@
         <v>2</v>
       </c>
       <c r="C9" s="3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D9" s="3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E9" s="3">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G9" s="3">
         <v>30</v>
@@ -1047,22 +1064,22 @@
         <v>1</v>
       </c>
       <c r="J9" s="8">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="K9" s="8">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L9" s="8">
         <v>1</v>
       </c>
       <c r="M9" s="8">
-        <v>1220</v>
+        <v>1251</v>
       </c>
       <c r="N9" s="8">
-        <v>32017</v>
+        <v>32932</v>
       </c>
       <c r="O9" s="8">
-        <v>60</v>
+        <v>90</v>
       </c>
     </row>
     <row r="10" spans="2:15">
@@ -1070,16 +1087,16 @@
         <v>2</v>
       </c>
       <c r="C10" s="3">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D10" s="3">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E10" s="3">
-        <v>90</v>
+        <v>120</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G10" s="3">
         <v>30</v>
@@ -1091,22 +1108,22 @@
         <v>1</v>
       </c>
       <c r="J10" s="8">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="K10" s="8">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L10" s="8">
         <v>1</v>
       </c>
       <c r="M10" s="8">
-        <v>1251</v>
+        <v>1282</v>
       </c>
       <c r="N10" s="8">
-        <v>32932</v>
+        <v>33847</v>
       </c>
       <c r="O10" s="8">
-        <v>90</v>
+        <v>120</v>
       </c>
     </row>
     <row r="11" spans="2:15">
@@ -1114,16 +1131,16 @@
         <v>2</v>
       </c>
       <c r="C11" s="3">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D11" s="3">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E11" s="3">
-        <v>120</v>
+        <v>150</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="G11" s="3">
         <v>30</v>
@@ -1135,22 +1152,22 @@
         <v>1</v>
       </c>
       <c r="J11" s="8">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="K11" s="8">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L11" s="8">
         <v>1</v>
       </c>
       <c r="M11" s="8">
-        <v>1282</v>
+        <v>1313</v>
       </c>
       <c r="N11" s="8">
-        <v>33847</v>
+        <v>34762</v>
       </c>
       <c r="O11" s="8">
-        <v>120</v>
+        <v>150</v>
       </c>
     </row>
     <row r="12" spans="2:15">
@@ -1158,16 +1175,16 @@
         <v>2</v>
       </c>
       <c r="C12" s="3">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D12" s="3">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E12" s="3">
-        <v>150</v>
+        <v>180</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G12" s="3">
         <v>30</v>
@@ -1179,22 +1196,22 @@
         <v>1</v>
       </c>
       <c r="J12" s="8">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="K12" s="8">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L12" s="8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M12" s="8">
-        <v>1313</v>
+        <v>1344</v>
       </c>
       <c r="N12" s="8">
-        <v>34762</v>
+        <v>38138</v>
       </c>
       <c r="O12" s="8">
-        <v>150</v>
+        <v>180</v>
       </c>
     </row>
     <row r="13" spans="2:15">
@@ -1202,16 +1219,16 @@
         <v>2</v>
       </c>
       <c r="C13" s="3">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D13" s="3">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E13" s="3">
-        <v>180</v>
+        <v>210</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G13" s="3">
         <v>30</v>
@@ -1223,22 +1240,22 @@
         <v>1</v>
       </c>
       <c r="J13" s="8">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="K13" s="8">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L13" s="8">
         <v>2</v>
       </c>
       <c r="M13" s="8">
-        <v>1344</v>
+        <v>1375</v>
       </c>
       <c r="N13" s="8">
-        <v>38138</v>
+        <v>39053</v>
       </c>
       <c r="O13" s="8">
-        <v>180</v>
+        <v>210</v>
       </c>
     </row>
     <row r="14" spans="2:15">
@@ -1246,16 +1263,16 @@
         <v>2</v>
       </c>
       <c r="C14" s="3">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D14" s="3">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E14" s="3">
-        <v>210</v>
+        <v>240</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="G14" s="3">
         <v>30</v>
@@ -1267,22 +1284,22 @@
         <v>1</v>
       </c>
       <c r="J14" s="8">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="K14" s="8">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="L14" s="8">
         <v>2</v>
       </c>
       <c r="M14" s="8">
-        <v>1375</v>
+        <v>1406</v>
       </c>
       <c r="N14" s="8">
-        <v>39053</v>
+        <v>39968</v>
       </c>
       <c r="O14" s="8">
-        <v>210</v>
+        <v>240</v>
       </c>
     </row>
     <row r="15" spans="2:15">
@@ -1290,16 +1307,16 @@
         <v>2</v>
       </c>
       <c r="C15" s="3">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D15" s="3">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E15" s="3">
-        <v>240</v>
+        <v>270</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G15" s="3">
         <v>30</v>
@@ -1311,22 +1328,22 @@
         <v>1</v>
       </c>
       <c r="J15" s="8">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="K15" s="8">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="L15" s="8">
         <v>2</v>
       </c>
       <c r="M15" s="8">
-        <v>1406</v>
+        <v>1437</v>
       </c>
       <c r="N15" s="8">
-        <v>39968</v>
+        <v>40883</v>
       </c>
       <c r="O15" s="8">
-        <v>240</v>
+        <v>270</v>
       </c>
     </row>
     <row r="16" spans="2:15">
@@ -1334,16 +1351,16 @@
         <v>2</v>
       </c>
       <c r="C16" s="3">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D16" s="3">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E16" s="3">
-        <v>270</v>
+        <v>300</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G16" s="3">
         <v>30</v>
@@ -1355,22 +1372,22 @@
         <v>1</v>
       </c>
       <c r="J16" s="8">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="K16" s="8">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="L16" s="8">
         <v>2</v>
       </c>
       <c r="M16" s="8">
-        <v>1437</v>
+        <v>1468</v>
       </c>
       <c r="N16" s="8">
-        <v>40883</v>
+        <v>41798</v>
       </c>
       <c r="O16" s="8">
-        <v>270</v>
+        <v>300</v>
       </c>
     </row>
     <row r="17" spans="2:15">
@@ -1378,16 +1395,16 @@
         <v>2</v>
       </c>
       <c r="C17" s="3">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D17" s="3">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E17" s="3">
-        <v>300</v>
+        <v>330</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G17" s="3">
         <v>30</v>
@@ -1399,22 +1416,22 @@
         <v>1</v>
       </c>
       <c r="J17" s="8">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="K17" s="8">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="L17" s="8">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M17" s="8">
-        <v>1468</v>
+        <v>1499</v>
       </c>
       <c r="N17" s="8">
-        <v>41798</v>
+        <v>45174</v>
       </c>
       <c r="O17" s="8">
-        <v>300</v>
+        <v>330</v>
       </c>
     </row>
     <row r="18" spans="2:15">
@@ -1422,16 +1439,16 @@
         <v>2</v>
       </c>
       <c r="C18" s="3">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D18" s="3">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E18" s="3">
-        <v>330</v>
+        <v>360</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="G18" s="3">
         <v>30</v>
@@ -1443,66 +1460,66 @@
         <v>1</v>
       </c>
       <c r="J18" s="8">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="K18" s="8">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="L18" s="8">
         <v>3</v>
       </c>
-      <c r="M18" s="8">
-        <v>1499</v>
+      <c r="M18" s="9">
+        <v>1530</v>
       </c>
       <c r="N18" s="8">
-        <v>45174</v>
+        <v>46089</v>
       </c>
       <c r="O18" s="8">
-        <v>330</v>
+        <v>360</v>
       </c>
     </row>
     <row r="19" spans="2:15">
       <c r="B19" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C19" s="3">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="D19" s="3">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="E19" s="3">
-        <v>360</v>
+        <v>40</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="G19" s="3">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="H19" s="8">
         <v>1</v>
       </c>
-      <c r="I19" s="8">
-        <v>1</v>
+      <c r="I19" s="9">
+        <v>0</v>
       </c>
       <c r="J19" s="8">
-        <v>72</v>
-      </c>
-      <c r="K19" s="8">
-        <v>12</v>
+        <v>8</v>
+      </c>
+      <c r="K19" s="9" t="s">
+        <v>38</v>
       </c>
       <c r="L19" s="8">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M19" s="9" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="N19" s="8">
-        <v>46089</v>
+        <v>352</v>
       </c>
       <c r="O19" s="8">
-        <v>360</v>
+        <v>40</v>
       </c>
     </row>
     <row r="20" spans="2:15">
@@ -1510,7 +1527,7 @@
         <v>3</v>
       </c>
       <c r="C20" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D20" s="3">
         <v>1</v>
@@ -1519,31 +1536,31 @@
         <v>40</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G20" s="3">
         <v>40</v>
       </c>
       <c r="H20" s="8">
-        <v>1</v>
-      </c>
-      <c r="I20" s="9">
-        <v>0</v>
+        <v>2</v>
+      </c>
+      <c r="I20" s="9" t="s">
+        <v>38</v>
       </c>
       <c r="J20" s="8">
         <v>8</v>
       </c>
-      <c r="K20" s="9" t="s">
-        <v>41</v>
+      <c r="K20" s="8">
+        <v>1</v>
       </c>
       <c r="L20" s="8">
         <v>1</v>
       </c>
-      <c r="M20" s="9" t="s">
-        <v>44</v>
+      <c r="M20" s="8">
+        <v>45</v>
       </c>
       <c r="N20" s="8">
-        <v>352</v>
+        <v>1489</v>
       </c>
       <c r="O20" s="8">
         <v>40</v>
@@ -1554,7 +1571,7 @@
         <v>3</v>
       </c>
       <c r="C21" s="3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D21" s="3">
         <v>1</v>
@@ -1572,7 +1589,7 @@
         <v>2</v>
       </c>
       <c r="I21" s="9" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="J21" s="8">
         <v>8</v>
@@ -1584,10 +1601,10 @@
         <v>1</v>
       </c>
       <c r="M21" s="8">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="N21" s="8">
-        <v>1489</v>
+        <v>1137</v>
       </c>
       <c r="O21" s="8">
         <v>40</v>
@@ -1598,25 +1615,25 @@
         <v>3</v>
       </c>
       <c r="C22" s="3">
+        <v>4</v>
+      </c>
+      <c r="D22" s="3">
+        <v>1</v>
+      </c>
+      <c r="E22" s="3">
+        <v>40</v>
+      </c>
+      <c r="F22" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="G22" s="3">
+        <v>40</v>
+      </c>
+      <c r="H22" s="8">
         <v>3</v>
       </c>
-      <c r="D22" s="3">
-        <v>1</v>
-      </c>
-      <c r="E22" s="3">
-        <v>40</v>
-      </c>
-      <c r="F22" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="G22" s="3">
-        <v>40</v>
-      </c>
-      <c r="H22" s="8">
-        <v>2</v>
-      </c>
       <c r="I22" s="9" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="J22" s="8">
         <v>8</v>
@@ -1628,10 +1645,10 @@
         <v>1</v>
       </c>
       <c r="M22" s="8">
-        <v>43</v>
+        <v>193</v>
       </c>
       <c r="N22" s="8">
-        <v>1137</v>
+        <v>3577</v>
       </c>
       <c r="O22" s="8">
         <v>40</v>
@@ -1642,7 +1659,7 @@
         <v>3</v>
       </c>
       <c r="C23" s="3">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D23" s="3">
         <v>1</v>
@@ -1657,10 +1674,10 @@
         <v>40</v>
       </c>
       <c r="H23" s="8">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I23" s="9" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="J23" s="8">
         <v>8</v>
@@ -1672,10 +1689,10 @@
         <v>1</v>
       </c>
       <c r="M23" s="8">
-        <v>193</v>
+        <v>157</v>
       </c>
       <c r="N23" s="8">
-        <v>3577</v>
+        <v>2573</v>
       </c>
       <c r="O23" s="8">
         <v>40</v>
@@ -1686,7 +1703,7 @@
         <v>3</v>
       </c>
       <c r="C24" s="3">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D24" s="3">
         <v>1</v>
@@ -1695,7 +1712,7 @@
         <v>40</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G24" s="3">
         <v>40</v>
@@ -1703,8 +1720,8 @@
       <c r="H24" s="8">
         <v>2</v>
       </c>
-      <c r="I24" s="9" t="s">
-        <v>41</v>
+      <c r="I24" s="8">
+        <v>2</v>
       </c>
       <c r="J24" s="8">
         <v>8</v>
@@ -1716,10 +1733,10 @@
         <v>1</v>
       </c>
       <c r="M24" s="8">
-        <v>157</v>
+        <v>128</v>
       </c>
       <c r="N24" s="8">
-        <v>2573</v>
+        <v>3496</v>
       </c>
       <c r="O24" s="8">
         <v>40</v>
@@ -1730,7 +1747,7 @@
         <v>3</v>
       </c>
       <c r="C25" s="3">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D25" s="3">
         <v>1</v>
@@ -1739,7 +1756,7 @@
         <v>40</v>
       </c>
       <c r="F25" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G25" s="3">
         <v>40</v>
@@ -1760,10 +1777,10 @@
         <v>1</v>
       </c>
       <c r="M25" s="8">
-        <v>128</v>
+        <v>136</v>
       </c>
       <c r="N25" s="8">
-        <v>3496</v>
+        <v>3951</v>
       </c>
       <c r="O25" s="8">
         <v>40</v>
@@ -1774,7 +1791,7 @@
         <v>3</v>
       </c>
       <c r="C26" s="3">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D26" s="3">
         <v>1</v>
@@ -1783,16 +1800,16 @@
         <v>40</v>
       </c>
       <c r="F26" s="4" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="G26" s="3">
         <v>40</v>
       </c>
-      <c r="H26" s="8">
-        <v>2</v>
+      <c r="H26" s="9" t="s">
+        <v>35</v>
       </c>
       <c r="I26" s="8">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J26" s="8">
         <v>8</v>
@@ -1804,10 +1821,10 @@
         <v>1</v>
       </c>
       <c r="M26" s="8">
-        <v>136</v>
+        <v>288</v>
       </c>
       <c r="N26" s="8">
-        <v>3951</v>
+        <v>7964</v>
       </c>
       <c r="O26" s="8">
         <v>40</v>
@@ -1818,7 +1835,7 @@
         <v>3</v>
       </c>
       <c r="C27" s="3">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D27" s="3">
         <v>1</v>
@@ -1827,16 +1844,16 @@
         <v>40</v>
       </c>
       <c r="F27" s="4" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="G27" s="3">
         <v>40</v>
       </c>
       <c r="H27" s="9" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="I27" s="8">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="J27" s="8">
         <v>8</v>
@@ -1848,10 +1865,10 @@
         <v>1</v>
       </c>
       <c r="M27" s="8">
-        <v>288</v>
+        <v>315</v>
       </c>
       <c r="N27" s="8">
-        <v>7964</v>
+        <v>7763</v>
       </c>
       <c r="O27" s="8">
         <v>40</v>
@@ -1862,7 +1879,7 @@
         <v>3</v>
       </c>
       <c r="C28" s="3">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D28" s="3">
         <v>1</v>
@@ -1871,16 +1888,16 @@
         <v>40</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="G28" s="3">
         <v>40</v>
       </c>
       <c r="H28" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="I28" s="8">
-        <v>19</v>
+        <v>37</v>
+      </c>
+      <c r="I28" s="9" t="s">
+        <v>38</v>
       </c>
       <c r="J28" s="8">
         <v>8</v>
@@ -1892,10 +1909,10 @@
         <v>1</v>
       </c>
       <c r="M28" s="8">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="N28" s="8">
-        <v>7763</v>
+        <v>8314</v>
       </c>
       <c r="O28" s="8">
         <v>40</v>
@@ -1906,7 +1923,7 @@
         <v>3</v>
       </c>
       <c r="C29" s="3">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D29" s="3">
         <v>1</v>
@@ -1915,16 +1932,16 @@
         <v>40</v>
       </c>
       <c r="F29" s="4" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="G29" s="3">
         <v>40</v>
       </c>
       <c r="H29" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="I29" s="9" t="s">
-        <v>41</v>
+        <v>36</v>
+      </c>
+      <c r="I29" s="8">
+        <v>19</v>
       </c>
       <c r="J29" s="8">
         <v>8</v>
@@ -1936,10 +1953,10 @@
         <v>1</v>
       </c>
       <c r="M29" s="8">
-        <v>317</v>
+        <v>433</v>
       </c>
       <c r="N29" s="8">
-        <v>8314</v>
+        <v>11917</v>
       </c>
       <c r="O29" s="8">
         <v>40</v>
@@ -1947,10 +1964,10 @@
     </row>
     <row r="30" spans="2:15">
       <c r="B30" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C30" s="3">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="D30" s="3">
         <v>1</v>
@@ -1959,16 +1976,16 @@
         <v>40</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="G30" s="3">
         <v>40</v>
       </c>
-      <c r="H30" s="9" t="s">
-        <v>39</v>
+      <c r="H30" s="8">
+        <v>1</v>
       </c>
       <c r="I30" s="8">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="J30" s="8">
         <v>8</v>
@@ -1980,10 +1997,10 @@
         <v>1</v>
       </c>
       <c r="M30" s="8">
-        <v>433</v>
+        <v>1189</v>
       </c>
       <c r="N30" s="8">
-        <v>11917</v>
+        <v>31102</v>
       </c>
       <c r="O30" s="8">
         <v>40</v>
@@ -1994,16 +2011,16 @@
         <v>4</v>
       </c>
       <c r="C31" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D31" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E31" s="3">
-        <v>40</v>
+        <v>80</v>
       </c>
       <c r="F31" s="4" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G31" s="3">
         <v>40</v>
@@ -2015,22 +2032,22 @@
         <v>1</v>
       </c>
       <c r="J31" s="8">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="K31" s="8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L31" s="8">
         <v>1</v>
       </c>
       <c r="M31" s="8">
-        <v>1189</v>
+        <v>1232</v>
       </c>
       <c r="N31" s="8">
-        <v>31102</v>
+        <v>32344</v>
       </c>
       <c r="O31" s="8">
-        <v>40</v>
+        <v>80</v>
       </c>
     </row>
     <row r="32" spans="2:15">
@@ -2038,16 +2055,16 @@
         <v>4</v>
       </c>
       <c r="C32" s="3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D32" s="3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E32" s="3">
-        <v>80</v>
+        <v>120</v>
       </c>
       <c r="F32" s="4" t="s">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="G32" s="3">
         <v>40</v>
@@ -2059,22 +2076,22 @@
         <v>1</v>
       </c>
       <c r="J32" s="8">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="K32" s="8">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L32" s="8">
         <v>1</v>
       </c>
       <c r="M32" s="8">
-        <v>1232</v>
+        <v>1272</v>
       </c>
       <c r="N32" s="8">
-        <v>32344</v>
+        <v>34449</v>
       </c>
       <c r="O32" s="8">
-        <v>80</v>
+        <v>120</v>
       </c>
     </row>
     <row r="33" spans="2:15">
@@ -2082,16 +2099,16 @@
         <v>4</v>
       </c>
       <c r="C33" s="3">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D33" s="3">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E33" s="3">
-        <v>120</v>
+        <v>160</v>
       </c>
       <c r="F33" s="4" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="G33" s="3">
         <v>40</v>
@@ -2103,22 +2120,22 @@
         <v>1</v>
       </c>
       <c r="J33" s="8">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="K33" s="8">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L33" s="8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M33" s="8">
-        <v>1272</v>
+        <v>1436</v>
       </c>
       <c r="N33" s="8">
-        <v>34449</v>
+        <v>36983</v>
       </c>
       <c r="O33" s="8">
-        <v>120</v>
+        <v>160</v>
       </c>
     </row>
     <row r="34" spans="2:15">
@@ -2126,16 +2143,16 @@
         <v>4</v>
       </c>
       <c r="C34" s="3">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D34" s="3">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E34" s="3">
-        <v>160</v>
+        <v>200</v>
       </c>
       <c r="F34" s="4" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="G34" s="3">
         <v>40</v>
@@ -2147,22 +2164,22 @@
         <v>1</v>
       </c>
       <c r="J34" s="8">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="K34" s="8">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L34" s="8">
         <v>2</v>
       </c>
       <c r="M34" s="8">
-        <v>1436</v>
+        <v>1499</v>
       </c>
       <c r="N34" s="8">
-        <v>36983</v>
+        <v>37666</v>
       </c>
       <c r="O34" s="8">
-        <v>160</v>
+        <v>200</v>
       </c>
     </row>
     <row r="35" spans="2:15">
@@ -2170,43 +2187,43 @@
         <v>4</v>
       </c>
       <c r="C35" s="3">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D35" s="3">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E35" s="3">
-        <v>200</v>
+        <v>280</v>
       </c>
       <c r="F35" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="G35" s="3">
+        <v>40</v>
+      </c>
+      <c r="H35" s="8">
+        <v>1</v>
+      </c>
+      <c r="I35" s="8">
+        <v>1</v>
+      </c>
+      <c r="J35" s="8">
+        <v>56</v>
+      </c>
+      <c r="K35" s="8">
         <v>7</v>
       </c>
-      <c r="G35" s="3">
-        <v>40</v>
-      </c>
-      <c r="H35" s="8">
-        <v>1</v>
-      </c>
-      <c r="I35" s="8">
-        <v>1</v>
-      </c>
-      <c r="J35" s="8">
-        <v>40</v>
-      </c>
-      <c r="K35" s="8">
-        <v>5</v>
-      </c>
       <c r="L35" s="8">
         <v>2</v>
       </c>
       <c r="M35" s="8">
-        <v>1499</v>
+        <v>1799</v>
       </c>
       <c r="N35" s="8">
-        <v>37666</v>
+        <v>44455</v>
       </c>
       <c r="O35" s="8">
-        <v>200</v>
+        <v>280</v>
       </c>
     </row>
     <row r="36" spans="2:15">
@@ -2214,16 +2231,16 @@
         <v>4</v>
       </c>
       <c r="C36" s="3">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D36" s="3">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E36" s="3">
-        <v>280</v>
+        <v>360</v>
       </c>
       <c r="F36" s="4" t="s">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="G36" s="3">
         <v>40</v>
@@ -2235,66 +2252,66 @@
         <v>1</v>
       </c>
       <c r="J36" s="8">
-        <v>56</v>
+        <v>72</v>
       </c>
       <c r="K36" s="8">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="L36" s="8">
         <v>2</v>
       </c>
       <c r="M36" s="8">
-        <v>1799</v>
+        <v>2039</v>
       </c>
       <c r="N36" s="8">
-        <v>44455</v>
+        <v>51994</v>
       </c>
       <c r="O36" s="8">
-        <v>280</v>
+        <v>360</v>
       </c>
     </row>
     <row r="37" spans="2:15">
       <c r="B37" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C37" s="3">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="D37" s="3">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="E37" s="3">
-        <v>360</v>
-      </c>
-      <c r="F37" s="4" t="s">
-        <v>18</v>
+        <v>0</v>
+      </c>
+      <c r="F37" s="4">
+        <v>0</v>
       </c>
       <c r="G37" s="3">
-        <v>40</v>
+        <v>357</v>
       </c>
       <c r="H37" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I37" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J37" s="8">
-        <v>72</v>
+        <v>0</v>
       </c>
       <c r="K37" s="8">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="L37" s="8">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M37" s="8">
-        <v>2039</v>
+        <v>0</v>
       </c>
       <c r="N37" s="8">
-        <v>51994</v>
+        <v>0</v>
       </c>
       <c r="O37" s="8">
-        <v>360</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38" spans="2:15">
@@ -2302,28 +2319,28 @@
         <v>5</v>
       </c>
       <c r="C38" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D38" s="3">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E38" s="3">
-        <v>30</v>
-      </c>
-      <c r="F38" s="4" t="s">
-        <v>11</v>
+        <v>0</v>
+      </c>
+      <c r="F38" s="4">
+        <v>0</v>
       </c>
       <c r="G38" s="3">
-        <v>40</v>
+        <v>357</v>
       </c>
       <c r="H38" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I38" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J38" s="8">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="K38" s="8">
         <v>1</v>
@@ -2332,13 +2349,13 @@
         <v>1</v>
       </c>
       <c r="M38" s="8">
-        <v>1189</v>
+        <v>0</v>
       </c>
       <c r="N38" s="8">
-        <v>31102</v>
+        <v>0</v>
       </c>
       <c r="O38" s="8">
-        <v>30</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39" spans="2:15">
@@ -2346,43 +2363,43 @@
         <v>5</v>
       </c>
       <c r="C39" s="3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D39" s="3">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E39" s="3">
-        <v>60</v>
-      </c>
-      <c r="F39" s="4" t="s">
-        <v>12</v>
+        <v>0</v>
+      </c>
+      <c r="F39" s="4">
+        <v>0</v>
       </c>
       <c r="G39" s="3">
-        <v>40</v>
+        <v>357</v>
       </c>
       <c r="H39" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I39" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J39" s="8">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="K39" s="8">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L39" s="8">
         <v>1</v>
       </c>
       <c r="M39" s="8">
-        <v>1220</v>
+        <v>0</v>
       </c>
       <c r="N39" s="8">
-        <v>32017</v>
+        <v>0</v>
       </c>
       <c r="O39" s="8">
-        <v>60</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40" spans="2:15">
@@ -2390,43 +2407,43 @@
         <v>5</v>
       </c>
       <c r="C40" s="3">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D40" s="3">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E40" s="3">
-        <v>90</v>
-      </c>
-      <c r="F40" s="4" t="s">
-        <v>29</v>
+        <v>0</v>
+      </c>
+      <c r="F40" s="4">
+        <v>0</v>
       </c>
       <c r="G40" s="3">
-        <v>40</v>
+        <v>357</v>
       </c>
       <c r="H40" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I40" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J40" s="8">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="K40" s="8">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L40" s="8">
         <v>1</v>
       </c>
       <c r="M40" s="8">
-        <v>1251</v>
+        <v>0</v>
       </c>
       <c r="N40" s="8">
-        <v>32932</v>
+        <v>0</v>
       </c>
       <c r="O40" s="8">
-        <v>90</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41" spans="2:15">
@@ -2434,87 +2451,43 @@
         <v>5</v>
       </c>
       <c r="C41" s="3">
+        <v>5</v>
+      </c>
+      <c r="D41" s="3">
         <v>4</v>
       </c>
-      <c r="D41" s="3">
-        <v>6</v>
-      </c>
       <c r="E41" s="3">
-        <v>180</v>
-      </c>
-      <c r="F41" s="4" t="s">
-        <v>8</v>
+        <v>0</v>
+      </c>
+      <c r="F41" s="4">
+        <v>0</v>
       </c>
       <c r="G41" s="3">
-        <v>40</v>
+        <v>357</v>
       </c>
       <c r="H41" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I41" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J41" s="8">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="K41" s="8">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="L41" s="8">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M41" s="8">
-        <v>1344</v>
+        <v>0</v>
       </c>
       <c r="N41" s="8">
-        <v>38138</v>
+        <v>0</v>
       </c>
       <c r="O41" s="8">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="42" spans="2:15">
-      <c r="B42" s="1">
-        <v>5</v>
-      </c>
-      <c r="C42" s="3">
-        <v>5</v>
-      </c>
-      <c r="D42" s="3">
-        <v>12</v>
-      </c>
-      <c r="E42" s="3">
-        <v>360</v>
-      </c>
-      <c r="F42" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="G42" s="3">
-        <v>40</v>
-      </c>
-      <c r="H42" s="8">
-        <v>1</v>
-      </c>
-      <c r="I42" s="8">
-        <v>1</v>
-      </c>
-      <c r="J42" s="8">
-        <v>72</v>
-      </c>
-      <c r="K42" s="8">
-        <v>12</v>
-      </c>
-      <c r="L42" s="8">
-        <v>3</v>
-      </c>
-      <c r="M42" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="N42" s="8">
-        <v>46089</v>
-      </c>
-      <c r="O42" s="8">
-        <v>360</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>